<commit_message>
Creacion de Tabla para Links de Formularios
</commit_message>
<xml_diff>
--- a/RH/Encuestas PESV/Informacion Encuesta.xlsx
+++ b/RH/Encuestas PESV/Informacion Encuesta.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pipea\OneDrive\Documentos\HIELO FOCA\RH\Encuestas PESV\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAF363E8-0B79-49FD-9B9F-22DDA84898DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD4E822D-9956-4A53-B622-34EEAB6DEE63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="30" windowWidth="20475" windowHeight="11490" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MOTO" sheetId="1" r:id="rId1"/>
-    <sheet name="CARRO" sheetId="2" r:id="rId2"/>
+    <sheet name="FORMULARIOS" sheetId="3" r:id="rId2"/>
+    <sheet name="CARRO" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="47">
   <si>
     <t>N°</t>
   </si>
@@ -48,39 +49,9 @@
     <t>CEDULA</t>
   </si>
   <si>
-    <t>N° Licencia Conduccion</t>
-  </si>
-  <si>
-    <t>Venc. Licencia Conduccion</t>
-  </si>
-  <si>
-    <t>Categoria</t>
-  </si>
-  <si>
-    <t>Placa</t>
-  </si>
-  <si>
-    <t>Restricciones de Licencia</t>
-  </si>
-  <si>
-    <t>Marca</t>
-  </si>
-  <si>
-    <t>Modelo</t>
-  </si>
-  <si>
-    <t>Tipo Vehiculo</t>
-  </si>
-  <si>
-    <t>N° Licencia Transito</t>
-  </si>
-  <si>
     <t>N° SOAT</t>
   </si>
   <si>
-    <t>N° Tecnomecanica</t>
-  </si>
-  <si>
     <t>PLACA</t>
   </si>
   <si>
@@ -175,6 +146,39 @@
   </si>
   <si>
     <t>NO APLICA</t>
+  </si>
+  <si>
+    <t>CONDUCTOR</t>
+  </si>
+  <si>
+    <t>FORMULARIO</t>
+  </si>
+  <si>
+    <t>MARCA</t>
+  </si>
+  <si>
+    <t>MODELO</t>
+  </si>
+  <si>
+    <t>TIPO VEHICULO</t>
+  </si>
+  <si>
+    <t>N° LICENCIA CONDUCCION</t>
+  </si>
+  <si>
+    <t>VENC. LICENCIA CONDUCCION</t>
+  </si>
+  <si>
+    <t>CATEGORIA</t>
+  </si>
+  <si>
+    <t>RESTRICCIONES DE LICENCIA</t>
+  </si>
+  <si>
+    <t>N° LICENCIA TRANSITO</t>
+  </si>
+  <si>
+    <t>N° TECNOMECANICA</t>
   </si>
 </sst>
 </file>
@@ -233,7 +237,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -274,12 +278,37 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Millares" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="24">
+  <dxfs count="31">
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -368,42 +397,58 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4EB8EF9E-F657-4A9B-97F3-DEAEEF4C48B6}" name="Conductores_Moto" displayName="Conductores_Moto" ref="B2:O11" totalsRowShown="0" headerRowDxfId="23" dataDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4EB8EF9E-F657-4A9B-97F3-DEAEEF4C48B6}" name="Conductores_Moto" displayName="Conductores_Moto" ref="B2:O11" totalsRowShown="0" headerRowDxfId="30" dataDxfId="21">
   <autoFilter ref="B2:O11" xr:uid="{4EB8EF9E-F657-4A9B-97F3-DEAEEF4C48B6}"/>
   <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{B05DCF9F-8C19-4B9F-891A-71C56544E8BB}" name="N°" dataDxfId="13">
+    <tableColumn id="1" xr3:uid="{B05DCF9F-8C19-4B9F-891A-71C56544E8BB}" name="N°" dataDxfId="20">
       <calculatedColumnFormula>ROW()-2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{04722251-E16B-483F-885A-8F5489E8C081}" name="NOMBRE" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{1667FFC6-5CFA-4D16-A2E8-789677901F04}" name="CEDULA" dataDxfId="11"/>
-    <tableColumn id="7" xr3:uid="{6BD6C41E-8ED0-4B3A-BA85-8817E7F84948}" name="Placa" dataDxfId="10"/>
-    <tableColumn id="9" xr3:uid="{04C1F34D-211E-404D-8881-7AD9C173F2CE}" name="Marca" dataDxfId="9"/>
-    <tableColumn id="10" xr3:uid="{21E5DA93-BBC1-4DA1-94FE-7873DAB21C12}" name="Modelo" dataDxfId="8"/>
-    <tableColumn id="11" xr3:uid="{613BFCEA-9818-44A5-BA5B-7E3022F70E5E}" name="Tipo Vehiculo" dataDxfId="7"/>
-    <tableColumn id="16" xr3:uid="{9C85E032-E7FA-449D-ADD8-BC273AB25810}" name="N° Licencia Conduccion" dataDxfId="6"/>
-    <tableColumn id="17" xr3:uid="{0EABB337-A64F-42DA-B479-1533888B4CF4}" name="Venc. Licencia Conduccion" dataDxfId="5"/>
-    <tableColumn id="18" xr3:uid="{79DBE90D-83C1-4AD8-8ECB-BBBF754F58F9}" name="Categoria" dataDxfId="4"/>
-    <tableColumn id="19" xr3:uid="{52861595-2667-4D03-ACDB-22A430E6757F}" name="Restricciones de Licencia" dataDxfId="3"/>
-    <tableColumn id="12" xr3:uid="{544A733D-86E5-45F0-8F5E-D5E1D1803CC4}" name="N° Licencia Transito" dataDxfId="2"/>
-    <tableColumn id="13" xr3:uid="{09A347FA-CD4A-4A8E-9BB1-882E6A9E78B3}" name="N° SOAT" dataDxfId="1"/>
-    <tableColumn id="14" xr3:uid="{F6D76FC3-D07A-4F3E-BCEA-BEF0EE802139}" name="N° Tecnomecanica" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{04722251-E16B-483F-885A-8F5489E8C081}" name="NOMBRE" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{1667FFC6-5CFA-4D16-A2E8-789677901F04}" name="CEDULA" dataDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{6BD6C41E-8ED0-4B3A-BA85-8817E7F84948}" name="PLACA" dataDxfId="17"/>
+    <tableColumn id="9" xr3:uid="{04C1F34D-211E-404D-8881-7AD9C173F2CE}" name="MARCA" dataDxfId="16"/>
+    <tableColumn id="10" xr3:uid="{21E5DA93-BBC1-4DA1-94FE-7873DAB21C12}" name="MODELO" dataDxfId="15"/>
+    <tableColumn id="11" xr3:uid="{613BFCEA-9818-44A5-BA5B-7E3022F70E5E}" name="TIPO VEHICULO" dataDxfId="14"/>
+    <tableColumn id="16" xr3:uid="{9C85E032-E7FA-449D-ADD8-BC273AB25810}" name="N° LICENCIA CONDUCCION" dataDxfId="13"/>
+    <tableColumn id="17" xr3:uid="{0EABB337-A64F-42DA-B479-1533888B4CF4}" name="VENC. LICENCIA CONDUCCION" dataDxfId="12"/>
+    <tableColumn id="18" xr3:uid="{79DBE90D-83C1-4AD8-8ECB-BBBF754F58F9}" name="CATEGORIA" dataDxfId="11"/>
+    <tableColumn id="19" xr3:uid="{52861595-2667-4D03-ACDB-22A430E6757F}" name="RESTRICCIONES DE LICENCIA" dataDxfId="10"/>
+    <tableColumn id="12" xr3:uid="{544A733D-86E5-45F0-8F5E-D5E1D1803CC4}" name="N° LICENCIA TRANSITO" dataDxfId="9"/>
+    <tableColumn id="13" xr3:uid="{09A347FA-CD4A-4A8E-9BB1-882E6A9E78B3}" name="N° SOAT" dataDxfId="8"/>
+    <tableColumn id="14" xr3:uid="{F6D76FC3-D07A-4F3E-BCEA-BEF0EE802139}" name="N° TECNOMECANICA" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium28" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2A0A5079-24CC-4112-AD76-C9290F2524CC}" name="Tabla2" displayName="Tabla2" ref="B2:G6" totalsRowShown="0" headerRowDxfId="22" dataDxfId="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{488A644D-9ED0-4366-AEC9-1D19BC94F4CA}" name="Formularios_Moto" displayName="Formularios_Moto" ref="B2:F11" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
+  <autoFilter ref="B2:F11" xr:uid="{488A644D-9ED0-4366-AEC9-1D19BC94F4CA}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{141E3A07-437E-4E13-A123-2FAA4976B715}" name="N°" dataDxfId="4">
+      <calculatedColumnFormula>ROW()-2</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="2" xr3:uid="{929476D5-F75C-4CD5-858C-5CC844CC79EC}" name="CONDUCTOR" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{0D3D7983-1DC0-4B9E-BA91-1CC6F3282C1D}" name="PLACA" dataDxfId="2"/>
+    <tableColumn id="9" xr3:uid="{FA36785A-0A16-4C69-B3FB-57D394FD2B3E}" name="MARCA" dataDxfId="1"/>
+    <tableColumn id="21" xr3:uid="{B4517C90-95DC-4162-A1F4-528D99A62D94}" name="FORMULARIO" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2A0A5079-24CC-4112-AD76-C9290F2524CC}" name="Tabla2" displayName="Tabla2" ref="B2:G6" totalsRowShown="0" headerRowDxfId="29" dataDxfId="22">
   <autoFilter ref="B2:G6" xr:uid="{2A0A5079-24CC-4112-AD76-C9290F2524CC}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{C3E741DD-FA44-4ADA-B312-DC357B39E691}" name="N°" dataDxfId="21">
+    <tableColumn id="1" xr3:uid="{C3E741DD-FA44-4ADA-B312-DC357B39E691}" name="N°" dataDxfId="28">
       <calculatedColumnFormula>ROW()-2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{4A828654-26E7-4BCB-9ADD-970633C742BB}" name="NOMBRE" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{83E3B254-B7D3-4BF5-8F39-973510DC4E4D}" name="PLACA" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{5B8AAE0D-2F8F-4F26-90CD-90B5213E4CC0}" name="N° Interno" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{85355C69-F663-447D-935C-A82B1BAC882A}" name="Area" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{14595361-A5D5-42ED-B318-C9BD12D23960}" name="Ciudad" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{4A828654-26E7-4BCB-9ADD-970633C742BB}" name="NOMBRE" dataDxfId="27"/>
+    <tableColumn id="3" xr3:uid="{83E3B254-B7D3-4BF5-8F39-973510DC4E4D}" name="PLACA" dataDxfId="26"/>
+    <tableColumn id="4" xr3:uid="{5B8AAE0D-2F8F-4F26-90CD-90B5213E4CC0}" name="N° Interno" dataDxfId="25"/>
+    <tableColumn id="5" xr3:uid="{85355C69-F663-447D-935C-A82B1BAC882A}" name="Area" dataDxfId="24"/>
+    <tableColumn id="6" xr3:uid="{14595361-A5D5-42ED-B318-C9BD12D23960}" name="Ciudad" dataDxfId="23"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium22" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -677,18 +722,18 @@
   <cols>
     <col min="2" max="2" width="8.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="33.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="26.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="29" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="27.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="29.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="32.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="30.7109375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="25.140625" customWidth="1"/>
     <col min="14" max="14" width="21" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="24" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:15" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -702,37 +747,37 @@
         <v>2</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>8</v>
+        <v>38</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>9</v>
+        <v>39</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="I2" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="M2" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="N2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="N2" s="4" t="s">
-        <v>12</v>
-      </c>
       <c r="O2" s="4" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="2:15" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -741,34 +786,34 @@
         <v>1</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="D3" s="4">
         <v>1075324543</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="G3" s="4">
         <v>2021</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="J3" s="9">
         <v>47213</v>
       </c>
       <c r="K3" s="4" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="L3" s="4" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="M3" s="4">
         <v>10021034204</v>
@@ -786,22 +831,22 @@
         <v>2</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="D4" s="5">
         <v>1075311763</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="G4" s="5">
         <v>2015</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="I4" s="5">
         <v>1075311763</v>
@@ -810,10 +855,10 @@
         <v>47370</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="L4" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="M4" s="6">
         <v>10018984694</v>
@@ -831,22 +876,22 @@
         <v>3</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="D5" s="1">
         <v>1075239239</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="G5" s="1">
         <v>2010</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="I5" s="1">
         <v>1075239239</v>
@@ -855,13 +900,13 @@
         <v>48246</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="M5" s="8" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="N5" s="12">
         <v>1308004373420000</v>
@@ -876,22 +921,22 @@
         <v>4</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="D6" s="1">
         <v>79411860</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="G6" s="1">
         <v>2024</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="I6" s="1">
         <v>79411860</v>
@@ -900,10 +945,10 @@
         <v>46186</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="M6" s="1">
         <v>10030491574</v>
@@ -921,22 +966,22 @@
         <v>5</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="D7" s="1">
         <v>1082214903</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="G7" s="1">
         <v>2008</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="I7" s="1">
         <v>1082214903</v>
@@ -945,10 +990,10 @@
         <v>48865</v>
       </c>
       <c r="K7" s="4" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="M7" s="1">
         <v>2656449</v>
@@ -966,22 +1011,22 @@
         <v>6</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="D8" s="1">
         <v>7725134</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="G8" s="1">
         <v>2011</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="I8" s="1">
         <v>7725134</v>
@@ -990,10 +1035,10 @@
         <v>48718</v>
       </c>
       <c r="K8" s="4" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="M8" s="1">
         <v>10018663952</v>
@@ -1011,22 +1056,22 @@
         <v>7</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="D9" s="1">
         <v>1148442390</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="G9" s="1">
         <v>2025</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="I9" s="1">
         <v>1148442390</v>
@@ -1035,10 +1080,10 @@
         <v>48231</v>
       </c>
       <c r="K9" s="4" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="M9" s="1">
         <v>10033684046</v>
@@ -1047,7 +1092,7 @@
         <v>40993052</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="2:15" x14ac:dyDescent="0.25">
@@ -1058,21 +1103,21 @@
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
       <c r="E10" s="1" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="G10" s="1">
         <v>2026</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
       <c r="K10" s="4" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="L10" s="1"/>
       <c r="M10" s="1">
@@ -1082,7 +1127,7 @@
         <v>4308006956131000</v>
       </c>
       <c r="O10" s="1" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="2:15" x14ac:dyDescent="0.25">
@@ -1093,21 +1138,21 @@
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
       <c r="E11" s="1" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="G11" s="1">
         <v>2026</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
       <c r="K11" s="4" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="L11" s="1"/>
       <c r="M11" s="1">
@@ -1117,7 +1162,7 @@
         <v>4308007126959000</v>
       </c>
       <c r="O11" s="1" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1138,12 +1183,189 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3D953E7-BFD9-4432-AE73-D0CDD23E1ADA}">
+  <dimension ref="B2:F11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B2" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B3" s="4">
+        <f t="shared" ref="B3:B4" si="0">ROW()-2</f>
+        <v>1</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="4"/>
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B4" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="4"/>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B5" s="3">
+        <f>ROW()-2</f>
+        <v>3</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" s="1"/>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B6" s="3">
+        <f>ROW()-2</f>
+        <v>4</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F6" s="1"/>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B7" s="3">
+        <f>ROW()-2</f>
+        <v>5</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" s="1"/>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B8" s="14">
+        <f>ROW()-2</f>
+        <v>6</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F8" s="1"/>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B9" s="14">
+        <f>ROW()-2</f>
+        <v>7</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F9" s="1"/>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B10" s="3">
+        <f>ROW()-2</f>
+        <v>8</v>
+      </c>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F10" s="1"/>
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B11" s="3">
+        <f>ROW()-2</f>
+        <v>9</v>
+      </c>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F11" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2A721AB-0148-41C4-B4F5-4C60F3EDF2E1}">
   <dimension ref="B2:G6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.7109375" bestFit="1" customWidth="1"/>
@@ -1158,16 +1380,16 @@
         <v>1</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="2:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Creacion de Vinculos para conductores
</commit_message>
<xml_diff>
--- a/RH/Encuestas PESV/Informacion Encuesta.xlsx
+++ b/RH/Encuestas PESV/Informacion Encuesta.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pipea\OneDrive\Documentos\HIELO FOCA\RH\Encuestas PESV\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD4E822D-9956-4A53-B622-34EEAB6DEE63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57140DBB-B77F-4054-A74C-6D5B81FD4DF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="30" windowWidth="20475" windowHeight="11490" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MOTO" sheetId="1" r:id="rId1"/>
@@ -37,8 +37,67 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Felipe Tovar Aviles</author>
+  </authors>
+  <commentList>
+    <comment ref="B8" authorId="0" shapeId="0" xr:uid="{A8B512D6-720F-4784-B160-035AC978034B}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Felipe Tovar Aviles:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+No conicide la licencia de transito presentada con la que esta registrada en el RUNT</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B9" authorId="0" shapeId="0" xr:uid="{C210537E-65EF-4264-9261-885F6A003FC1}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Felipe Tovar Aviles:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+SOAT VENCIDO
+</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="65">
   <si>
     <t>N°</t>
   </si>
@@ -151,9 +210,6 @@
     <t>CONDUCTOR</t>
   </si>
   <si>
-    <t>FORMULARIO</t>
-  </si>
-  <si>
     <t>MARCA</t>
   </si>
   <si>
@@ -179,6 +235,63 @@
   </si>
   <si>
     <t>N° TECNOMECANICA</t>
+  </si>
+  <si>
+    <t>CODIGO</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FORMULARIO MOTO: </t>
+  </si>
+  <si>
+    <t>FORMULARIO CARRO:</t>
+  </si>
+  <si>
+    <t>https://forms.gle/Qhk9jswMSuKSRXJC9</t>
+  </si>
+  <si>
+    <t>https://forms.gle/nV4Mp5DGBGCDpVoV8</t>
+  </si>
+  <si>
+    <t>FORMULARIOS</t>
+  </si>
+  <si>
+    <t>LINK</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.1224725918=CARLOS+ANDRES+CALDERON+VARGAS&amp;entry.1043732100=1075324543&amp;entry.1844146731=1508020348020941&amp;entry.2019467002=2029-04-05&amp;entry.2034385725=A2&amp;entry.1717299640=KXD64F&amp;entry.1644177803=NINGUNA&amp;entry.1623663502=BAJAJ&amp;entry.1795124056=2021&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=10021034204&amp;entry.1834591344=14289413182430&amp;entry.2070070149=180673854</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.1224725918=CRISTIAN+ANDRES+RICO+YULE&amp;entry.1043732100=1075311763&amp;entry.1844146731=1075311763&amp;entry.2019467002=2029-09-09&amp;entry.2034385725=A2&amp;entry.1717299640=SAE17D&amp;entry.1644177803=CONDUCIR+CON+LENTES&amp;entry.1623663502=AKT&amp;entry.1795124056=2015&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=10018984694&amp;entry.1834591344=4308006501614000&amp;entry.2070070149=179996307</t>
+  </si>
+  <si>
+    <t>VEHICULO</t>
+  </si>
+  <si>
+    <t>MOTO</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.1224725918=JOHN+ELKIN+RIOS+CORDOBA&amp;entry.1043732100=1075239239&amp;entry.1844146731=1075239239&amp;entry.2019467002=2032-02-02&amp;entry.2034385725=A2&amp;entry.1717299640=QTZ14B&amp;entry.1644177803=NINGUNA&amp;entry.1623663502=SUZUKI&amp;entry.1795124056=2010&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=4141049&amp;entry.1834591344=1308004373420000&amp;entry.2070070149=181663842</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.1224725918=JORGE+GONZALEZ+MARTINEZ&amp;entry.1043732100=79411860&amp;entry.1844146731=79411860&amp;entry.2019467002=2026-06-13&amp;entry.2034385725=A2&amp;entry.1717299640=VRR30G&amp;entry.1644177803=CONDUCIR+CON+LENTES&amp;entry.1623663502=SUZUKI&amp;entry.1795124056=2024&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=10030491574&amp;entry.1834591344=93868954&amp;entry.2070070149=185413046</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.1224725918=JOSE+WILLIAM+PE%C3%91A+GONZALEZ&amp;entry.1043732100=1082214903&amp;entry.1844146731=1082214903&amp;entry.2019467002=2033-10-13&amp;entry.2034385725=A2&amp;entry.1717299640=INX92B&amp;entry.1644177803=NINGUNA&amp;entry.1623663502=HONDA&amp;entry.1795124056=2008&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=2656449&amp;entry.1834591344=4308007922847000&amp;entry.2070070149=185049856</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.1717299640=RFL57H&amp;entry.1623663502=HERO&amp;entry.1795124056=2026&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=10035852978&amp;entry.1834591344=4308007126959000&amp;entry.2070070149=NO+APLICA</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.2034385725=A02&amp;entry.1717299640=REJ11H&amp;entry.1623663502=HERO&amp;entry.1795124056=2026&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=10034787944&amp;entry.1834591344=4308006956131000&amp;entry.2070070149=NO+APLICA</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.1224725918=CRISTIAN+DAVID+BRAVO+QUINTERO&amp;entry.1043732100=1148442390&amp;entry.1844146731=1148442390&amp;entry.2019467002=2032-01-18&amp;entry.2034385725=A2&amp;entry.1717299640=JGC42H&amp;entry.1644177803=NINGUNA&amp;entry.1623663502=BAJAJ&amp;entry.1795124056=2025&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=10033684046&amp;entry.1834591344=4308006927176000&amp;entry.2070070149=182958025</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.1224725918=MANOLO+MENZA+ESCOBAR&amp;entry.1043732100=7725134&amp;entry.1844146731=7725134&amp;entry.2019467002=2033-05-19&amp;entry.2034385725=A2&amp;entry.1717299640=MAC23C&amp;entry.1644177803=NINGUNA&amp;entry.1623663502=BAJAJ&amp;entry.1795124056=2011&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=10018663952&amp;entry.1834591344=4308006927176000&amp;entry.2070070149=182958025</t>
   </si>
 </sst>
 </file>
@@ -188,7 +301,7 @@
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -205,6 +318,42 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -233,60 +382,69 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Hipervínculo" xfId="2" builtinId="8"/>
     <cellStyle name="Millares" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="31">
+  <dxfs count="33">
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -325,31 +483,34 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -397,58 +558,60 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4EB8EF9E-F657-4A9B-97F3-DEAEEF4C48B6}" name="Conductores_Moto" displayName="Conductores_Moto" ref="B2:O11" totalsRowShown="0" headerRowDxfId="30" dataDxfId="21">
-  <autoFilter ref="B2:O11" xr:uid="{4EB8EF9E-F657-4A9B-97F3-DEAEEF4C48B6}"/>
-  <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{B05DCF9F-8C19-4B9F-891A-71C56544E8BB}" name="N°" dataDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4EB8EF9E-F657-4A9B-97F3-DEAEEF4C48B6}" name="Conductores_Moto" displayName="Conductores_Moto" ref="B2:P11" totalsRowShown="0" headerRowDxfId="32" dataDxfId="31">
+  <autoFilter ref="B2:P11" xr:uid="{4EB8EF9E-F657-4A9B-97F3-DEAEEF4C48B6}"/>
+  <tableColumns count="15">
+    <tableColumn id="1" xr3:uid="{B05DCF9F-8C19-4B9F-891A-71C56544E8BB}" name="N°" dataDxfId="30">
       <calculatedColumnFormula>ROW()-2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{04722251-E16B-483F-885A-8F5489E8C081}" name="NOMBRE" dataDxfId="19"/>
-    <tableColumn id="3" xr3:uid="{1667FFC6-5CFA-4D16-A2E8-789677901F04}" name="CEDULA" dataDxfId="18"/>
-    <tableColumn id="7" xr3:uid="{6BD6C41E-8ED0-4B3A-BA85-8817E7F84948}" name="PLACA" dataDxfId="17"/>
-    <tableColumn id="9" xr3:uid="{04C1F34D-211E-404D-8881-7AD9C173F2CE}" name="MARCA" dataDxfId="16"/>
-    <tableColumn id="10" xr3:uid="{21E5DA93-BBC1-4DA1-94FE-7873DAB21C12}" name="MODELO" dataDxfId="15"/>
-    <tableColumn id="11" xr3:uid="{613BFCEA-9818-44A5-BA5B-7E3022F70E5E}" name="TIPO VEHICULO" dataDxfId="14"/>
-    <tableColumn id="16" xr3:uid="{9C85E032-E7FA-449D-ADD8-BC273AB25810}" name="N° LICENCIA CONDUCCION" dataDxfId="13"/>
-    <tableColumn id="17" xr3:uid="{0EABB337-A64F-42DA-B479-1533888B4CF4}" name="VENC. LICENCIA CONDUCCION" dataDxfId="12"/>
-    <tableColumn id="18" xr3:uid="{79DBE90D-83C1-4AD8-8ECB-BBBF754F58F9}" name="CATEGORIA" dataDxfId="11"/>
-    <tableColumn id="19" xr3:uid="{52861595-2667-4D03-ACDB-22A430E6757F}" name="RESTRICCIONES DE LICENCIA" dataDxfId="10"/>
-    <tableColumn id="12" xr3:uid="{544A733D-86E5-45F0-8F5E-D5E1D1803CC4}" name="N° LICENCIA TRANSITO" dataDxfId="9"/>
-    <tableColumn id="13" xr3:uid="{09A347FA-CD4A-4A8E-9BB1-882E6A9E78B3}" name="N° SOAT" dataDxfId="8"/>
-    <tableColumn id="14" xr3:uid="{F6D76FC3-D07A-4F3E-BCEA-BEF0EE802139}" name="N° TECNOMECANICA" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{04722251-E16B-483F-885A-8F5489E8C081}" name="NOMBRE" dataDxfId="29"/>
+    <tableColumn id="3" xr3:uid="{1667FFC6-5CFA-4D16-A2E8-789677901F04}" name="CEDULA" dataDxfId="28"/>
+    <tableColumn id="7" xr3:uid="{6BD6C41E-8ED0-4B3A-BA85-8817E7F84948}" name="PLACA" dataDxfId="27"/>
+    <tableColumn id="9" xr3:uid="{04C1F34D-211E-404D-8881-7AD9C173F2CE}" name="MARCA" dataDxfId="26"/>
+    <tableColumn id="10" xr3:uid="{21E5DA93-BBC1-4DA1-94FE-7873DAB21C12}" name="MODELO" dataDxfId="25"/>
+    <tableColumn id="11" xr3:uid="{613BFCEA-9818-44A5-BA5B-7E3022F70E5E}" name="TIPO VEHICULO" dataDxfId="24"/>
+    <tableColumn id="16" xr3:uid="{9C85E032-E7FA-449D-ADD8-BC273AB25810}" name="N° LICENCIA CONDUCCION" dataDxfId="23"/>
+    <tableColumn id="17" xr3:uid="{0EABB337-A64F-42DA-B479-1533888B4CF4}" name="VENC. LICENCIA CONDUCCION" dataDxfId="22"/>
+    <tableColumn id="18" xr3:uid="{79DBE90D-83C1-4AD8-8ECB-BBBF754F58F9}" name="CATEGORIA" dataDxfId="21"/>
+    <tableColumn id="19" xr3:uid="{52861595-2667-4D03-ACDB-22A430E6757F}" name="RESTRICCIONES DE LICENCIA" dataDxfId="20"/>
+    <tableColumn id="12" xr3:uid="{544A733D-86E5-45F0-8F5E-D5E1D1803CC4}" name="N° LICENCIA TRANSITO" dataDxfId="19"/>
+    <tableColumn id="13" xr3:uid="{09A347FA-CD4A-4A8E-9BB1-882E6A9E78B3}" name="N° SOAT" dataDxfId="18"/>
+    <tableColumn id="14" xr3:uid="{F6D76FC3-D07A-4F3E-BCEA-BEF0EE802139}" name="N° TECNOMECANICA" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{FEC06E28-DF71-468A-9F6A-07BDE02B29EF}" name="CODIGO" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium28" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{488A644D-9ED0-4366-AEC9-1D19BC94F4CA}" name="Formularios_Moto" displayName="Formularios_Moto" ref="B2:F11" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
-  <autoFilter ref="B2:F11" xr:uid="{488A644D-9ED0-4366-AEC9-1D19BC94F4CA}"/>
-  <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{141E3A07-437E-4E13-A123-2FAA4976B715}" name="N°" dataDxfId="4">
-      <calculatedColumnFormula>ROW()-2</calculatedColumnFormula>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{488A644D-9ED0-4366-AEC9-1D19BC94F4CA}" name="Formularios_Moto" displayName="Formularios_Moto" ref="B6:G15" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
+  <autoFilter ref="B6:G15" xr:uid="{488A644D-9ED0-4366-AEC9-1D19BC94F4CA}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{141E3A07-437E-4E13-A123-2FAA4976B715}" name="N°" dataDxfId="13">
+      <calculatedColumnFormula>ROW()-6</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{929476D5-F75C-4CD5-858C-5CC844CC79EC}" name="CONDUCTOR" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{0D3D7983-1DC0-4B9E-BA91-1CC6F3282C1D}" name="PLACA" dataDxfId="2"/>
-    <tableColumn id="9" xr3:uid="{FA36785A-0A16-4C69-B3FB-57D394FD2B3E}" name="MARCA" dataDxfId="1"/>
-    <tableColumn id="21" xr3:uid="{B4517C90-95DC-4162-A1F4-528D99A62D94}" name="FORMULARIO" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{929476D5-F75C-4CD5-858C-5CC844CC79EC}" name="CONDUCTOR" dataDxfId="12"/>
+    <tableColumn id="7" xr3:uid="{0D3D7983-1DC0-4B9E-BA91-1CC6F3282C1D}" name="PLACA" dataDxfId="11"/>
+    <tableColumn id="9" xr3:uid="{FA36785A-0A16-4C69-B3FB-57D394FD2B3E}" name="MARCA" dataDxfId="10"/>
+    <tableColumn id="21" xr3:uid="{B4517C90-95DC-4162-A1F4-528D99A62D94}" name="LINK" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{C51A2751-FF3B-4E60-969D-B81446AB2AB4}" name="VEHICULO" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2A0A5079-24CC-4112-AD76-C9290F2524CC}" name="Tabla2" displayName="Tabla2" ref="B2:G6" totalsRowShown="0" headerRowDxfId="29" dataDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2A0A5079-24CC-4112-AD76-C9290F2524CC}" name="Tabla2" displayName="Tabla2" ref="B2:G6" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
   <autoFilter ref="B2:G6" xr:uid="{2A0A5079-24CC-4112-AD76-C9290F2524CC}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{C3E741DD-FA44-4ADA-B312-DC357B39E691}" name="N°" dataDxfId="28">
+    <tableColumn id="1" xr3:uid="{C3E741DD-FA44-4ADA-B312-DC357B39E691}" name="N°" dataDxfId="5">
       <calculatedColumnFormula>ROW()-2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{4A828654-26E7-4BCB-9ADD-970633C742BB}" name="NOMBRE" dataDxfId="27"/>
-    <tableColumn id="3" xr3:uid="{83E3B254-B7D3-4BF5-8F39-973510DC4E4D}" name="PLACA" dataDxfId="26"/>
-    <tableColumn id="4" xr3:uid="{5B8AAE0D-2F8F-4F26-90CD-90B5213E4CC0}" name="N° Interno" dataDxfId="25"/>
-    <tableColumn id="5" xr3:uid="{85355C69-F663-447D-935C-A82B1BAC882A}" name="Area" dataDxfId="24"/>
-    <tableColumn id="6" xr3:uid="{14595361-A5D5-42ED-B318-C9BD12D23960}" name="Ciudad" dataDxfId="23"/>
+    <tableColumn id="2" xr3:uid="{4A828654-26E7-4BCB-9ADD-970633C742BB}" name="NOMBRE" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{83E3B254-B7D3-4BF5-8F39-973510DC4E4D}" name="PLACA" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{5B8AAE0D-2F8F-4F26-90CD-90B5213E4CC0}" name="N° Interno" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{85355C69-F663-447D-935C-A82B1BAC882A}" name="Area" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{14595361-A5D5-42ED-B318-C9BD12D23960}" name="Ciudad" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium22" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -716,8 +879,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:O11"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="B2:P11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="8.5703125" bestFit="1" customWidth="1"/>
@@ -736,143 +899,152 @@
     <col min="15" max="15" width="24" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="4" t="s">
+    <row r="2" spans="2:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="H2" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="I2" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="J2" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="K2" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="L2" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="M2" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="N2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="O2" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="N2" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="O2" s="4" t="s">
+      <c r="P2" s="1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="2:15" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="4">
+    <row r="3" spans="2:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="1">
         <f t="shared" ref="B3:B4" si="0">ROW()-2</f>
         <v>1</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="1">
         <v>1075324543</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="4">
+      <c r="G3" s="1">
         <v>2021</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="I3" s="8" t="s">
+      <c r="I3" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="J3" s="9">
+      <c r="J3" s="6">
         <v>47213</v>
       </c>
-      <c r="K3" s="4" t="s">
+      <c r="K3" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="L3" s="4" t="s">
+      <c r="L3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="M3" s="4">
+      <c r="M3" s="1">
         <v>10021034204</v>
       </c>
-      <c r="N3" s="7">
+      <c r="N3" s="4">
         <v>14289413182430</v>
       </c>
-      <c r="O3" s="4">
+      <c r="O3" s="1">
         <v>180673854</v>
       </c>
-    </row>
-    <row r="4" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B4" s="4">
+      <c r="P3" s="1">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="2:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="1">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="2">
         <v>1075311763</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="2">
         <v>2015</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="H4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="I4" s="5">
+      <c r="I4" s="2">
         <v>1075311763</v>
       </c>
-      <c r="J4" s="10">
+      <c r="J4" s="7">
         <v>47370</v>
       </c>
-      <c r="K4" s="4" t="s">
+      <c r="K4" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="L4" s="5" t="s">
+      <c r="L4" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="M4" s="6">
+      <c r="M4" s="3">
         <v>10018984694</v>
       </c>
-      <c r="N4" s="7">
+      <c r="N4" s="4">
         <v>4308006501614000</v>
       </c>
-      <c r="O4" s="4">
+      <c r="O4" s="1">
         <v>179996307</v>
       </c>
-    </row>
-    <row r="5" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B5" s="3">
-        <f>ROW()-2</f>
+      <c r="P4" s="1">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="5" spans="2:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="1">
+        <f t="shared" ref="B5:B11" si="1">ROW()-2</f>
         <v>3</v>
       </c>
       <c r="C5" s="1" t="s">
@@ -890,34 +1062,37 @@
       <c r="G5" s="1">
         <v>2010</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" s="1" t="s">
         <v>17</v>
       </c>
       <c r="I5" s="1">
         <v>1075239239</v>
       </c>
-      <c r="J5" s="11">
+      <c r="J5" s="6">
         <v>48246</v>
       </c>
-      <c r="K5" s="4" t="s">
+      <c r="K5" s="1" t="s">
         <v>30</v>
       </c>
       <c r="L5" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="M5" s="8" t="s">
+      <c r="M5" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="N5" s="12">
+      <c r="N5" s="4">
         <v>1308004373420000</v>
       </c>
       <c r="O5" s="1">
         <v>181663842</v>
       </c>
-    </row>
-    <row r="6" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B6" s="3">
-        <f>ROW()-2</f>
+      <c r="P5" s="1">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6" spans="2:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="1">
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="C6" s="1" t="s">
@@ -941,13 +1116,13 @@
       <c r="I6" s="1">
         <v>79411860</v>
       </c>
-      <c r="J6" s="11">
+      <c r="J6" s="6">
         <v>46186</v>
       </c>
-      <c r="K6" s="4" t="s">
+      <c r="K6" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="L6" s="5" t="s">
+      <c r="L6" s="2" t="s">
         <v>32</v>
       </c>
       <c r="M6" s="1">
@@ -959,10 +1134,13 @@
       <c r="O6" s="1">
         <v>185413046</v>
       </c>
-    </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B7" s="3">
-        <f>ROW()-2</f>
+      <c r="P6" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" spans="2:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="1">
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="C7" s="1" t="s">
@@ -986,10 +1164,10 @@
       <c r="I7" s="1">
         <v>1082214903</v>
       </c>
-      <c r="J7" s="11">
+      <c r="J7" s="6">
         <v>48865</v>
       </c>
-      <c r="K7" s="4" t="s">
+      <c r="K7" s="1" t="s">
         <v>30</v>
       </c>
       <c r="L7" s="1" t="s">
@@ -998,16 +1176,19 @@
       <c r="M7" s="1">
         <v>2656449</v>
       </c>
-      <c r="N7" s="12">
+      <c r="N7" s="4">
         <v>4308007922847000</v>
       </c>
       <c r="O7" s="1">
         <v>185049856</v>
       </c>
-    </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B8" s="13">
-        <f>ROW()-2</f>
+      <c r="P7" s="1">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="8" spans="2:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="8">
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="C8" s="1" t="s">
@@ -1031,10 +1212,10 @@
       <c r="I8" s="1">
         <v>7725134</v>
       </c>
-      <c r="J8" s="11">
+      <c r="J8" s="6">
         <v>48718</v>
       </c>
-      <c r="K8" s="4" t="s">
+      <c r="K8" s="1" t="s">
         <v>30</v>
       </c>
       <c r="L8" s="1" t="s">
@@ -1043,16 +1224,19 @@
       <c r="M8" s="1">
         <v>10018663952</v>
       </c>
-      <c r="N8" s="12">
+      <c r="N8" s="4">
         <v>4308006927176000</v>
       </c>
       <c r="O8" s="1">
         <v>182958025</v>
       </c>
-    </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B9" s="13">
-        <f>ROW()-2</f>
+      <c r="P8" s="1">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="9" spans="2:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="8">
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
       <c r="C9" s="1" t="s">
@@ -1076,10 +1260,10 @@
       <c r="I9" s="1">
         <v>1148442390</v>
       </c>
-      <c r="J9" s="11">
+      <c r="J9" s="6">
         <v>48231</v>
       </c>
-      <c r="K9" s="4" t="s">
+      <c r="K9" s="1" t="s">
         <v>30</v>
       </c>
       <c r="L9" s="1" t="s">
@@ -1094,10 +1278,13 @@
       <c r="O9" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B10" s="3">
-        <f>ROW()-2</f>
+      <c r="P9" s="1">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="10" spans="2:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="1">
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
       <c r="C10" s="1"/>
@@ -1116,23 +1303,24 @@
       </c>
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
-      <c r="K10" s="4" t="s">
+      <c r="K10" s="1" t="s">
         <v>30</v>
       </c>
       <c r="L10" s="1"/>
       <c r="M10" s="1">
         <v>10034787944</v>
       </c>
-      <c r="N10" s="12">
+      <c r="N10" s="4">
         <v>4308006956131000</v>
       </c>
       <c r="O10" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B11" s="3">
-        <f>ROW()-2</f>
+      <c r="P10" s="1"/>
+    </row>
+    <row r="11" spans="2:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="1">
+        <f t="shared" si="1"/>
         <v>9</v>
       </c>
       <c r="C11" s="1"/>
@@ -1151,19 +1339,20 @@
       </c>
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
-      <c r="K11" s="4" t="s">
+      <c r="K11" s="1" t="s">
         <v>30</v>
       </c>
       <c r="L11" s="1"/>
       <c r="M11" s="1">
         <v>10035852978</v>
       </c>
-      <c r="N11" s="12">
+      <c r="N11" s="4">
         <v>4308007126959000</v>
       </c>
       <c r="O11" s="1" t="s">
         <v>35</v>
       </c>
+      <c r="P11" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -1176,185 +1365,288 @@
   <ignoredErrors>
     <ignoredError sqref="I3 M5" numberStoredAsText="1"/>
   </ignoredErrors>
+  <legacyDrawing r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3D953E7-BFD9-4432-AE73-D0CDD23E1ADA}">
-  <dimension ref="B2:F11"/>
+  <dimension ref="B1:G18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="7.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="33.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="14.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B2" s="4" t="s">
+    <row r="1" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+    </row>
+    <row r="3" spans="2:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="9"/>
+      <c r="C3" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="E3" s="15"/>
+      <c r="F3" s="15"/>
+    </row>
+    <row r="4" spans="2:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="9"/>
+      <c r="C4" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B6" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C6" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="F2" s="4" t="s">
+      <c r="E6" s="1" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B3" s="4">
-        <f t="shared" ref="B3:B4" si="0">ROW()-2</f>
+      <c r="F6" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B7" s="1">
+        <f t="shared" ref="B7:B15" si="0">ROW()-6</f>
         <v>1</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C7" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="4"/>
-    </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B4" s="4">
+      <c r="F7" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B8" s="1">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E8" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="4"/>
-    </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B5" s="3">
-        <f>ROW()-2</f>
+      <c r="F8" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B9" s="1">
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D9" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E9" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F5" s="1"/>
-    </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B6" s="3">
-        <f>ROW()-2</f>
+      <c r="F9" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="G9" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B10" s="1">
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D10" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E10" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F6" s="1"/>
-    </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B7" s="3">
-        <f>ROW()-2</f>
+      <c r="F10" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B11" s="1">
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C11" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D11" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E11" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F7" s="1"/>
-    </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B8" s="14">
-        <f>ROW()-2</f>
+      <c r="F11" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="G11" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B12" s="1">
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C12" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="D12" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="E12" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F8" s="1"/>
-    </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B9" s="14">
-        <f>ROW()-2</f>
+      <c r="F12" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="G12" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B13" s="1">
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C13" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="D13" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="E13" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F9" s="1"/>
-    </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B10" s="3">
-        <f>ROW()-2</f>
+      <c r="F13" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="G13" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B14" s="1">
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1" t="s">
+      <c r="C14" s="1"/>
+      <c r="D14" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E14" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F10" s="1"/>
-    </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B11" s="3">
-        <f>ROW()-2</f>
+      <c r="F14" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="G14" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="15" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B15" s="1">
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1" t="s">
+      <c r="C15" s="1"/>
+      <c r="D15" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="E15" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F11" s="1"/>
+      <c r="F15" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="G15" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="18" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F18" s="13"/>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="D3:F3"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="B1:F1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="D3" r:id="rId1" xr:uid="{9BECD8A1-6318-4374-94A7-2E9DE4FB7962}"/>
+    <hyperlink ref="D4" r:id="rId2" xr:uid="{AE28B26A-4B85-4BFA-A2B5-F4749951DC43}"/>
+    <hyperlink ref="F7" r:id="rId3" display="https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.1224725918=CARLOS+ANDRES+CALDERON+VARGAS&amp;entry.1043732100=1075324543&amp;entry.1844146731=1508020348020941&amp;entry.2019467002=2029-04-05&amp;entry.2034385725=A2&amp;entry.1717299640=KXD64F&amp;entry.1644177803=NINGUNA&amp;entry.1623663502=BAJAJ&amp;entry.1795124056=2021&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=10021034204&amp;entry.1834591344=14289413182430&amp;entry.2070070149=180673854" xr:uid="{AF8286B2-332B-4A17-B4C2-81AC9BE2C36C}"/>
+    <hyperlink ref="F8" r:id="rId4" display="https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.1224725918=CRISTIAN+ANDRES+RICO+YULE&amp;entry.1043732100=1075311763&amp;entry.1844146731=1075311763&amp;entry.2019467002=2029-09-09&amp;entry.2034385725=A2&amp;entry.1717299640=SAE17D&amp;entry.1644177803=CONDUCIR+CON+LENTES&amp;entry.1623663502=AKT&amp;entry.1795124056=2015&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=10018984694&amp;entry.1834591344=4308006501614000&amp;entry.2070070149=179996307" xr:uid="{73DC7536-7A36-412E-BD95-07A4FA1E536A}"/>
+    <hyperlink ref="F9" r:id="rId5" display="https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.1224725918=JOHN+ELKIN+RIOS+CORDOBA&amp;entry.1043732100=1075239239&amp;entry.1844146731=1075239239&amp;entry.2019467002=2032-02-02&amp;entry.2034385725=A2&amp;entry.1717299640=QTZ14B&amp;entry.1644177803=NINGUNA&amp;entry.1623663502=SUZUKI&amp;entry.1795124056=2010&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=4141049&amp;entry.1834591344=1308004373420000&amp;entry.2070070149=181663842" xr:uid="{7EF8F12E-FC1D-48F7-AF02-3B9BAFDA6CC9}"/>
+    <hyperlink ref="F10" r:id="rId6" display="https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.1224725918=JORGE+GONZALEZ+MARTINEZ&amp;entry.1043732100=79411860&amp;entry.1844146731=79411860&amp;entry.2019467002=2026-06-13&amp;entry.2034385725=A2&amp;entry.1717299640=VRR30G&amp;entry.1644177803=CONDUCIR+CON+LENTES&amp;entry.1623663502=SUZUKI&amp;entry.1795124056=2024&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=10030491574&amp;entry.1834591344=93868954&amp;entry.2070070149=185413046" xr:uid="{BD685723-6BD0-44DB-8B65-070F957E6220}"/>
+    <hyperlink ref="F11" r:id="rId7" display="https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.1224725918=JOSE+WILLIAM+PE%C3%91A+GONZALEZ&amp;entry.1043732100=1082214903&amp;entry.1844146731=1082214903&amp;entry.2019467002=2033-10-13&amp;entry.2034385725=A2&amp;entry.1717299640=INX92B&amp;entry.1644177803=NINGUNA&amp;entry.1623663502=HONDA&amp;entry.1795124056=2008&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=2656449&amp;entry.1834591344=4308007922847000&amp;entry.2070070149=185049856" xr:uid="{BEB06002-E60C-4548-A35B-95DB0362073B}"/>
+    <hyperlink ref="F13" r:id="rId8" display="https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.1224725918=CRISTIAN+DAVID+BRAVO+QUINTERO&amp;entry.1043732100=1148442390&amp;entry.1844146731=1148442390&amp;entry.2019467002=2032-01-18&amp;entry.2034385725=A2&amp;entry.1717299640=JGC42H&amp;entry.1644177803=NINGUNA&amp;entry.1623663502=BAJAJ&amp;entry.1795124056=2025&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=10033684046&amp;entry.1834591344=4308006927176000&amp;entry.2070070149=182958025" xr:uid="{CEF3CBCA-29DB-4D71-BA12-9B4344EB199A}"/>
+    <hyperlink ref="F15" r:id="rId9" display="https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.1717299640=RFL57H&amp;entry.1623663502=HERO&amp;entry.1795124056=2026&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=10035852978&amp;entry.1834591344=4308007126959000&amp;entry.2070070149=NO+APLICA" xr:uid="{1CC841B5-FDC4-480F-B9E9-9309C02C666B}"/>
+    <hyperlink ref="F14" r:id="rId10" display="https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.2034385725=A02&amp;entry.1717299640=REJ11H&amp;entry.1623663502=HERO&amp;entry.1795124056=2026&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=10034787944&amp;entry.1834591344=4308006956131000&amp;entry.2070070149=NO+APLICA" xr:uid="{06C2681C-13F8-4FBD-8ACE-624C074BB4DB}"/>
+    <hyperlink ref="F12" r:id="rId11" display="https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.1224725918=MANOLO+MENZA+ESCOBAR&amp;entry.1043732100=7725134&amp;entry.1844146731=7725134&amp;entry.2019467002=2033-05-19&amp;entry.2034385725=A2&amp;entry.1717299640=MAC23C&amp;entry.1644177803=NINGUNA&amp;entry.1623663502=BAJAJ&amp;entry.1795124056=2011&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=10018663952&amp;entry.1834591344=4308006927176000&amp;entry.2070070149=182958025" xr:uid="{D0F562E5-FA00-4E2F-B20D-133B4A54E888}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId12"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId13"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1393,11 +1685,11 @@
       </c>
     </row>
     <row r="3" spans="2:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="2">
+      <c r="B3" s="1">
         <f t="shared" ref="B3:B5" si="0">ROW()-2</f>
         <v>1</v>
       </c>
-      <c r="C3" s="2"/>
+      <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -1426,7 +1718,7 @@
       <c r="G5" s="1"/>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B6" s="3">
+      <c r="B6" s="1">
         <f>ROW()-2</f>
         <v>4</v>
       </c>

</xml_diff>

<commit_message>
Actualizacion de datos para conductores faltantes
</commit_message>
<xml_diff>
--- a/RH/Encuestas PESV/Informacion Encuesta.xlsx
+++ b/RH/Encuestas PESV/Informacion Encuesta.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pipea\OneDrive\Documentos\HIELO FOCA\RH\Encuestas PESV\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57140DBB-B77F-4054-A74C-6D5B81FD4DF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AD043E8-FCC5-4030-A100-3B6FC6883E29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="90" yWindow="30" windowWidth="20400" windowHeight="11490" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MOTO" sheetId="1" r:id="rId1"/>
@@ -97,7 +97,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="82">
   <si>
     <t>N°</t>
   </si>
@@ -282,16 +282,67 @@
     <t>https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.1224725918=JOSE+WILLIAM+PE%C3%91A+GONZALEZ&amp;entry.1043732100=1082214903&amp;entry.1844146731=1082214903&amp;entry.2019467002=2033-10-13&amp;entry.2034385725=A2&amp;entry.1717299640=INX92B&amp;entry.1644177803=NINGUNA&amp;entry.1623663502=HONDA&amp;entry.1795124056=2008&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=2656449&amp;entry.1834591344=4308007922847000&amp;entry.2070070149=185049856</t>
   </si>
   <si>
-    <t>https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.1717299640=RFL57H&amp;entry.1623663502=HERO&amp;entry.1795124056=2026&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=10035852978&amp;entry.1834591344=4308007126959000&amp;entry.2070070149=NO+APLICA</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.2034385725=A02&amp;entry.1717299640=REJ11H&amp;entry.1623663502=HERO&amp;entry.1795124056=2026&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=10034787944&amp;entry.1834591344=4308006956131000&amp;entry.2070070149=NO+APLICA</t>
-  </si>
-  <si>
     <t>https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.1224725918=CRISTIAN+DAVID+BRAVO+QUINTERO&amp;entry.1043732100=1148442390&amp;entry.1844146731=1148442390&amp;entry.2019467002=2032-01-18&amp;entry.2034385725=A2&amp;entry.1717299640=JGC42H&amp;entry.1644177803=NINGUNA&amp;entry.1623663502=BAJAJ&amp;entry.1795124056=2025&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=10033684046&amp;entry.1834591344=4308006927176000&amp;entry.2070070149=182958025</t>
   </si>
   <si>
     <t>https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.1224725918=MANOLO+MENZA+ESCOBAR&amp;entry.1043732100=7725134&amp;entry.1844146731=7725134&amp;entry.2019467002=2033-05-19&amp;entry.2034385725=A2&amp;entry.1717299640=MAC23C&amp;entry.1644177803=NINGUNA&amp;entry.1623663502=BAJAJ&amp;entry.1795124056=2011&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=10018663952&amp;entry.1834591344=4308006927176000&amp;entry.2070070149=182958025</t>
+  </si>
+  <si>
+    <t>ANDRES MAURICIO CASTAÑEDA</t>
+  </si>
+  <si>
+    <t>JOSE ESTEIVY CUELLAR</t>
+  </si>
+  <si>
+    <t>LPY606</t>
+  </si>
+  <si>
+    <t>CHEVROLET</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/forms/d/e/1FAIpQLSevgNeiR-8AjnIN2DoSnpwTsaSIJOMFFwSNsHfTME17o5u0Dw/viewform?usp=pp_url&amp;entry.1966606223=LPY606&amp;entry.705265064=COMERCIAL&amp;entry.45486543=NEIVA</t>
+  </si>
+  <si>
+    <t>CARRO</t>
+  </si>
+  <si>
+    <t>GRK715</t>
+  </si>
+  <si>
+    <t>JAC</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/forms/d/e/1FAIpQLSevgNeiR-8AjnIN2DoSnpwTsaSIJOMFFwSNsHfTME17o5u0Dw/viewform?usp=pp_url&amp;entry.1966606223=GRK715&amp;entry.705265064=COMERCIAL&amp;entry.45486543=NEIVA</t>
+  </si>
+  <si>
+    <t>CSX344</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/forms/d/e/1FAIpQLSevgNeiR-8AjnIN2DoSnpwTsaSIJOMFFwSNsHfTME17o5u0Dw/viewform?usp=pp_url&amp;entry.1966606223=CSX344&amp;entry.705265064=COMERCIAL&amp;entry.45486543=NEIVA</t>
+  </si>
+  <si>
+    <t>BKC394</t>
+  </si>
+  <si>
+    <t>HYUNDAI</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/forms/d/e/1FAIpQLSevgNeiR-8AjnIN2DoSnpwTsaSIJOMFFwSNsHfTME17o5u0Dw/viewform?usp=pp_url&amp;entry.1966606223=BKC394&amp;entry.705265064=COMERCIAL&amp;entry.45486543=NEIVA</t>
+  </si>
+  <si>
+    <t>NHU059</t>
+  </si>
+  <si>
+    <t>FOTON</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/forms/d/e/1FAIpQLSevgNeiR-8AjnIN2DoSnpwTsaSIJOMFFwSNsHfTME17o5u0Dw/viewform?usp=pp_url&amp;entry.1966606223=NHU059&amp;entry.705265064=COMERCIAL&amp;entry.45486543=NEIVA</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.1224725918=ANDRES+MAURICIO+CASTA%C3%91EDA&amp;entry.1043732100=1003813474&amp;entry.1844146731=1003813474&amp;entry.2019467002=2029-06-08&amp;entry.2034385725=A2&amp;entry.1717299640=REJ11H&amp;entry.1644177803=CONDUCIR+CON+LENTES&amp;entry.1623663502=HERO&amp;entry.1795124056=2026&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=10034787944&amp;entry.1834591344=4308006956131000&amp;entry.2070070149=NO+APLICA</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.1224725918=JOSE+ESTEIVY+CUELLAR&amp;entry.1043732100=7725542&amp;entry.1844146731=7725542&amp;entry.2019467002=2034-06-09&amp;entry.2034385725=A2&amp;entry.1717299640=RFL57H&amp;entry.1644177803=NINGUNA&amp;entry.1623663502=HERO&amp;entry.1795124056=2026&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=10035852978&amp;entry.1834591344=4308007126959000&amp;entry.2070070149=NO+APLICA</t>
   </si>
 </sst>
 </file>
@@ -301,7 +352,7 @@
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -358,6 +409,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -387,7 +445,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -425,7 +483,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -433,6 +490,12 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -584,34 +647,34 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{488A644D-9ED0-4366-AEC9-1D19BC94F4CA}" name="Formularios_Moto" displayName="Formularios_Moto" ref="B6:G15" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
-  <autoFilter ref="B6:G15" xr:uid="{488A644D-9ED0-4366-AEC9-1D19BC94F4CA}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{488A644D-9ED0-4366-AEC9-1D19BC94F4CA}" name="Formularios_Moto" displayName="Formularios_Moto" ref="B6:G20" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
+  <autoFilter ref="B6:G20" xr:uid="{488A644D-9ED0-4366-AEC9-1D19BC94F4CA}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{141E3A07-437E-4E13-A123-2FAA4976B715}" name="N°" dataDxfId="13">
+    <tableColumn id="1" xr3:uid="{141E3A07-437E-4E13-A123-2FAA4976B715}" name="N°" dataDxfId="5">
       <calculatedColumnFormula>ROW()-6</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{929476D5-F75C-4CD5-858C-5CC844CC79EC}" name="CONDUCTOR" dataDxfId="12"/>
-    <tableColumn id="7" xr3:uid="{0D3D7983-1DC0-4B9E-BA91-1CC6F3282C1D}" name="PLACA" dataDxfId="11"/>
-    <tableColumn id="9" xr3:uid="{FA36785A-0A16-4C69-B3FB-57D394FD2B3E}" name="MARCA" dataDxfId="10"/>
-    <tableColumn id="21" xr3:uid="{B4517C90-95DC-4162-A1F4-528D99A62D94}" name="LINK" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{C51A2751-FF3B-4E60-969D-B81446AB2AB4}" name="VEHICULO" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{929476D5-F75C-4CD5-858C-5CC844CC79EC}" name="CONDUCTOR" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{0D3D7983-1DC0-4B9E-BA91-1CC6F3282C1D}" name="PLACA" dataDxfId="3"/>
+    <tableColumn id="9" xr3:uid="{FA36785A-0A16-4C69-B3FB-57D394FD2B3E}" name="MARCA" dataDxfId="2"/>
+    <tableColumn id="21" xr3:uid="{B4517C90-95DC-4162-A1F4-528D99A62D94}" name="LINK" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{C51A2751-FF3B-4E60-969D-B81446AB2AB4}" name="VEHICULO" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2A0A5079-24CC-4112-AD76-C9290F2524CC}" name="Tabla2" displayName="Tabla2" ref="B2:G6" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2A0A5079-24CC-4112-AD76-C9290F2524CC}" name="Tabla2" displayName="Tabla2" ref="B2:G6" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
   <autoFilter ref="B2:G6" xr:uid="{2A0A5079-24CC-4112-AD76-C9290F2524CC}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{C3E741DD-FA44-4ADA-B312-DC357B39E691}" name="N°" dataDxfId="5">
+    <tableColumn id="1" xr3:uid="{C3E741DD-FA44-4ADA-B312-DC357B39E691}" name="N°" dataDxfId="13">
       <calculatedColumnFormula>ROW()-2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{4A828654-26E7-4BCB-9ADD-970633C742BB}" name="NOMBRE" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{83E3B254-B7D3-4BF5-8F39-973510DC4E4D}" name="PLACA" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{5B8AAE0D-2F8F-4F26-90CD-90B5213E4CC0}" name="N° Interno" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{85355C69-F663-447D-935C-A82B1BAC882A}" name="Area" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{14595361-A5D5-42ED-B318-C9BD12D23960}" name="Ciudad" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{4A828654-26E7-4BCB-9ADD-970633C742BB}" name="NOMBRE" dataDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{83E3B254-B7D3-4BF5-8F39-973510DC4E4D}" name="PLACA" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{5B8AAE0D-2F8F-4F26-90CD-90B5213E4CC0}" name="N° Interno" dataDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{85355C69-F663-447D-935C-A82B1BAC882A}" name="Area" dataDxfId="9"/>
+    <tableColumn id="6" xr3:uid="{14595361-A5D5-42ED-B318-C9BD12D23960}" name="Ciudad" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium22" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1287,8 +1350,12 @@
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
+      <c r="C10" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D10" s="16">
+        <v>1003813474</v>
+      </c>
       <c r="E10" s="1" t="s">
         <v>27</v>
       </c>
@@ -1301,12 +1368,18 @@
       <c r="H10" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="I10" s="1"/>
-      <c r="J10" s="1"/>
+      <c r="I10" s="16">
+        <v>1003813474</v>
+      </c>
+      <c r="J10" s="17">
+        <v>47277</v>
+      </c>
       <c r="K10" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="L10" s="1"/>
+      <c r="L10" s="2" t="s">
+        <v>32</v>
+      </c>
       <c r="M10" s="1">
         <v>10034787944</v>
       </c>
@@ -1316,15 +1389,21 @@
       <c r="O10" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="P10" s="1"/>
+      <c r="P10" s="1">
+        <v>56</v>
+      </c>
     </row>
     <row r="11" spans="2:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="1">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
+      <c r="C11" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="D11" s="16">
+        <v>7725542</v>
+      </c>
       <c r="E11" s="1" t="s">
         <v>29</v>
       </c>
@@ -1337,12 +1416,18 @@
       <c r="H11" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="I11" s="1"/>
-      <c r="J11" s="1"/>
+      <c r="I11" s="16">
+        <v>7725542</v>
+      </c>
+      <c r="J11" s="6">
+        <v>49104</v>
+      </c>
       <c r="K11" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="L11" s="1"/>
+      <c r="L11" s="1" t="s">
+        <v>33</v>
+      </c>
       <c r="M11" s="1">
         <v>10035852978</v>
       </c>
@@ -1352,7 +1437,9 @@
       <c r="O11" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="P11" s="1"/>
+      <c r="P11" s="1">
+        <v>55</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -1362,19 +1449,20 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
   <ignoredErrors>
     <ignoredError sqref="I3 M5" numberStoredAsText="1"/>
   </ignoredErrors>
-  <legacyDrawing r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3D953E7-BFD9-4432-AE73-D0CDD23E1ADA}">
-  <dimension ref="B1:G18"/>
+  <dimension ref="B1:G20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="7.7109375" bestFit="1" customWidth="1"/>
@@ -1386,35 +1474,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="16" t="s">
+      <c r="B1" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
     </row>
     <row r="3" spans="2:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="9"/>
       <c r="C3" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="D3" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
     </row>
     <row r="4" spans="2:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="9"/>
       <c r="C4" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="E4" s="15"/>
-      <c r="F4" s="15"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
@@ -1438,7 +1526,7 @@
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B7" s="1">
-        <f t="shared" ref="B7:B15" si="0">ROW()-6</f>
+        <f t="shared" ref="B7:B20" si="0">ROW()-6</f>
         <v>1</v>
       </c>
       <c r="C7" s="1" t="s">
@@ -1556,7 +1644,7 @@
         <v>9</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G12" s="12" t="s">
         <v>57</v>
@@ -1577,7 +1665,7 @@
         <v>9</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="G13" s="12" t="s">
         <v>57</v>
@@ -1588,7 +1676,9 @@
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C14" s="1"/>
+      <c r="C14" s="1" t="s">
+        <v>63</v>
+      </c>
       <c r="D14" s="1" t="s">
         <v>27</v>
       </c>
@@ -1596,7 +1686,7 @@
         <v>28</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>62</v>
+        <v>80</v>
       </c>
       <c r="G14" s="12" t="s">
         <v>57</v>
@@ -1607,7 +1697,9 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C15" s="1"/>
+      <c r="C15" s="1" t="s">
+        <v>64</v>
+      </c>
       <c r="D15" s="1" t="s">
         <v>29</v>
       </c>
@@ -1615,14 +1707,106 @@
         <v>28</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>61</v>
+        <v>81</v>
       </c>
       <c r="G15" s="12" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="18" spans="6:6" x14ac:dyDescent="0.25">
-      <c r="F18" s="13"/>
+    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B16" s="1">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="F16" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B17" s="1">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="F17" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B18" s="1">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B19" s="1">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B20" s="1">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="F20" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>68</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1638,15 +1822,19 @@
     <hyperlink ref="F9" r:id="rId5" display="https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.1224725918=JOHN+ELKIN+RIOS+CORDOBA&amp;entry.1043732100=1075239239&amp;entry.1844146731=1075239239&amp;entry.2019467002=2032-02-02&amp;entry.2034385725=A2&amp;entry.1717299640=QTZ14B&amp;entry.1644177803=NINGUNA&amp;entry.1623663502=SUZUKI&amp;entry.1795124056=2010&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=4141049&amp;entry.1834591344=1308004373420000&amp;entry.2070070149=181663842" xr:uid="{7EF8F12E-FC1D-48F7-AF02-3B9BAFDA6CC9}"/>
     <hyperlink ref="F10" r:id="rId6" display="https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.1224725918=JORGE+GONZALEZ+MARTINEZ&amp;entry.1043732100=79411860&amp;entry.1844146731=79411860&amp;entry.2019467002=2026-06-13&amp;entry.2034385725=A2&amp;entry.1717299640=VRR30G&amp;entry.1644177803=CONDUCIR+CON+LENTES&amp;entry.1623663502=SUZUKI&amp;entry.1795124056=2024&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=10030491574&amp;entry.1834591344=93868954&amp;entry.2070070149=185413046" xr:uid="{BD685723-6BD0-44DB-8B65-070F957E6220}"/>
     <hyperlink ref="F11" r:id="rId7" display="https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.1224725918=JOSE+WILLIAM+PE%C3%91A+GONZALEZ&amp;entry.1043732100=1082214903&amp;entry.1844146731=1082214903&amp;entry.2019467002=2033-10-13&amp;entry.2034385725=A2&amp;entry.1717299640=INX92B&amp;entry.1644177803=NINGUNA&amp;entry.1623663502=HONDA&amp;entry.1795124056=2008&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=2656449&amp;entry.1834591344=4308007922847000&amp;entry.2070070149=185049856" xr:uid="{BEB06002-E60C-4548-A35B-95DB0362073B}"/>
-    <hyperlink ref="F13" r:id="rId8" display="https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.1224725918=CRISTIAN+DAVID+BRAVO+QUINTERO&amp;entry.1043732100=1148442390&amp;entry.1844146731=1148442390&amp;entry.2019467002=2032-01-18&amp;entry.2034385725=A2&amp;entry.1717299640=JGC42H&amp;entry.1644177803=NINGUNA&amp;entry.1623663502=BAJAJ&amp;entry.1795124056=2025&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=10033684046&amp;entry.1834591344=4308006927176000&amp;entry.2070070149=182958025" xr:uid="{CEF3CBCA-29DB-4D71-BA12-9B4344EB199A}"/>
-    <hyperlink ref="F15" r:id="rId9" display="https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.1717299640=RFL57H&amp;entry.1623663502=HERO&amp;entry.1795124056=2026&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=10035852978&amp;entry.1834591344=4308007126959000&amp;entry.2070070149=NO+APLICA" xr:uid="{1CC841B5-FDC4-480F-B9E9-9309C02C666B}"/>
-    <hyperlink ref="F14" r:id="rId10" display="https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.2034385725=A02&amp;entry.1717299640=REJ11H&amp;entry.1623663502=HERO&amp;entry.1795124056=2026&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=10034787944&amp;entry.1834591344=4308006956131000&amp;entry.2070070149=NO+APLICA" xr:uid="{06C2681C-13F8-4FBD-8ACE-624C074BB4DB}"/>
-    <hyperlink ref="F12" r:id="rId11" display="https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.1224725918=MANOLO+MENZA+ESCOBAR&amp;entry.1043732100=7725134&amp;entry.1844146731=7725134&amp;entry.2019467002=2033-05-19&amp;entry.2034385725=A2&amp;entry.1717299640=MAC23C&amp;entry.1644177803=NINGUNA&amp;entry.1623663502=BAJAJ&amp;entry.1795124056=2011&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=10018663952&amp;entry.1834591344=4308006927176000&amp;entry.2070070149=182958025" xr:uid="{D0F562E5-FA00-4E2F-B20D-133B4A54E888}"/>
+    <hyperlink ref="F12" r:id="rId8" display="https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.1224725918=MANOLO+MENZA+ESCOBAR&amp;entry.1043732100=7725134&amp;entry.1844146731=7725134&amp;entry.2019467002=2033-05-19&amp;entry.2034385725=A2&amp;entry.1717299640=MAC23C&amp;entry.1644177803=NINGUNA&amp;entry.1623663502=BAJAJ&amp;entry.1795124056=2011&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=10018663952&amp;entry.1834591344=4308006927176000&amp;entry.2070070149=182958025" xr:uid="{D0F562E5-FA00-4E2F-B20D-133B4A54E888}"/>
+    <hyperlink ref="F13" r:id="rId9" display="https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.1224725918=CRISTIAN+DAVID+BRAVO+QUINTERO&amp;entry.1043732100=1148442390&amp;entry.1844146731=1148442390&amp;entry.2019467002=2032-01-18&amp;entry.2034385725=A2&amp;entry.1717299640=JGC42H&amp;entry.1644177803=NINGUNA&amp;entry.1623663502=BAJAJ&amp;entry.1795124056=2025&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=10033684046&amp;entry.1834591344=4308006927176000&amp;entry.2070070149=182958025" xr:uid="{CEF3CBCA-29DB-4D71-BA12-9B4344EB199A}"/>
+    <hyperlink ref="F16" r:id="rId10" xr:uid="{1AD8AD98-D2F5-40C7-94FF-8BD9CF8F450A}"/>
+    <hyperlink ref="F17" r:id="rId11" xr:uid="{FB220C76-C943-497E-A099-3EA7C597E4C8}"/>
+    <hyperlink ref="F19" r:id="rId12" xr:uid="{0364E726-A77F-4386-BFBB-8B97C6AB3D5A}"/>
+    <hyperlink ref="F20" r:id="rId13" xr:uid="{E9E8496C-8DF3-4775-B747-7B340F5A45F1}"/>
+    <hyperlink ref="F14" r:id="rId14" display="https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.1224725918=ANDRES+MAURICIO+CASTA%C3%91EDA&amp;entry.1043732100=1003813474&amp;entry.1844146731=1003813474&amp;entry.2019467002=2029-06-08&amp;entry.2034385725=A2&amp;entry.1717299640=REJ11H&amp;entry.1644177803=CONDUCIR+CON+LENTES&amp;entry.1623663502=HERO&amp;entry.1795124056=2026&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=10034787944&amp;entry.1834591344=4308006956131000&amp;entry.2070070149=NO+APLICA" xr:uid="{C0A2638F-5F63-4CC6-9B0A-A1589A0136B3}"/>
+    <hyperlink ref="F15" r:id="rId15" display="https://docs.google.com/forms/d/e/1FAIpQLSf2pJ73zFe6TAay0oYKYYPF68Im7rg3dvWmxiA1LSkIXWRcrA/viewform?usp=pp_url&amp;entry.1224725918=JOSE+ESTEIVY+CUELLAR&amp;entry.1043732100=7725542&amp;entry.1844146731=7725542&amp;entry.2019467002=2034-06-09&amp;entry.2034385725=A2&amp;entry.1717299640=RFL57H&amp;entry.1644177803=NINGUNA&amp;entry.1623663502=HERO&amp;entry.1795124056=2026&amp;entry.818059440=Motocicleta+Igual+o+Inferior+a+125+cc&amp;entry.1881975723=10035852978&amp;entry.1834591344=4308007126959000&amp;entry.2070070149=NO+APLICA" xr:uid="{3A61AF9A-3383-4D4C-A04F-234D2799AB10}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId12"/>
+  <pageSetup orientation="portrait" verticalDpi="360" r:id="rId16"/>
   <tableParts count="1">
-    <tablePart r:id="rId13"/>
+    <tablePart r:id="rId17"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>